<commit_message>
Deploy latest storefront with persistent data
</commit_message>
<xml_diff>
--- a/public/product-import-template.xlsx
+++ b/public/product-import-template.xlsx
@@ -397,119 +397,129 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="38.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>賣場名稱</v>
+        <v>??</v>
       </c>
       <c r="B1" t="str">
-        <v>商品名稱</v>
+        <v>???</v>
       </c>
       <c r="C1" t="str">
-        <v>商品說明</v>
+        <v>????</v>
       </c>
       <c r="D1" t="str">
-        <v>商品圖片網址</v>
+        <v>????</v>
       </c>
       <c r="E1" t="str">
-        <v>款式</v>
+        <v>??????</v>
       </c>
       <c r="F1" t="str">
-        <v>品項條碼</v>
+        <v>??</v>
       </c>
       <c r="G1" t="str">
-        <v>售價</v>
+        <v>????</v>
       </c>
       <c r="H1" t="str">
-        <v>數量</v>
+        <v>??</v>
       </c>
       <c r="I1" t="str">
-        <v>品項圖片網址</v>
+        <v>??</v>
       </c>
       <c r="J1" t="str">
-        <v>是否上架</v>
+        <v>??????</v>
+      </c>
+      <c r="K1" t="str">
+        <v>????</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>夏季拖鞋賣場</v>
+        <v>??</v>
       </c>
       <c r="B2" t="str">
-        <v>雲朵厚底拖鞋</v>
+        <v>????</v>
       </c>
       <c r="C2" t="str">
-        <v>柔軟厚底，適合居家與外出。</v>
+        <v>??????</v>
       </c>
       <c r="D2" t="str">
-        <v>https://example.com/product.jpg</v>
+        <v>?????????????</v>
       </c>
       <c r="E2" t="str">
-        <v>白色 / 24cm</v>
+        <v/>
       </c>
       <c r="F2" t="str">
+        <v>?? / 24cm</v>
+      </c>
+      <c r="G2" t="str">
         <v>SLP-CW-24</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>390</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>20</v>
       </c>
-      <c r="I2" t="str">
-        <v>https://example.com/white-24.jpg</v>
-      </c>
       <c r="J2" t="str">
-        <v>是</v>
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>?</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>夏季拖鞋賣場</v>
+        <v>??</v>
       </c>
       <c r="B3" t="str">
-        <v>雲朵厚底拖鞋</v>
+        <v>????</v>
       </c>
       <c r="C3" t="str">
-        <v>柔軟厚底，適合居家與外出。</v>
+        <v>??????</v>
       </c>
       <c r="D3" t="str">
-        <v>https://example.com/product.jpg</v>
+        <v>????????????????</v>
       </c>
       <c r="E3" t="str">
-        <v>白色 / 25cm</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>SLP-CW-25</v>
-      </c>
-      <c r="G3">
-        <v>390</v>
+        <v>?? / M</v>
+      </c>
+      <c r="G3" t="str">
+        <v>SLP-BL-M</v>
       </c>
       <c r="H3">
-        <v>20</v>
-      </c>
-      <c r="I3" t="str">
-        <v>https://example.com/white-25.jpg</v>
+        <v>250</v>
+      </c>
+      <c r="I3">
+        <v>14</v>
       </c>
       <c r="J3" t="str">
-        <v>是</v>
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>?</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>